<commit_message>
Record final Google indexing submissions
</commit_message>
<xml_diff>
--- a/outputs/seo-handover-2026-09-11/Pelit_Park_SEO_Baseline_and_Handover_2026-09-11.xlsx
+++ b/outputs/seo-handover-2026-09-11/Pelit_Park_SEO_Baseline_and_Handover_2026-09-11.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb4eaa4d615fd4dc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Queries" sheetId="2" r:id="Rb10ce49a65ec4a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="3" r:id="R3a7c2b9418f94467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Countries" sheetId="4" r:id="R65615e513e6b47ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language Paths" sheetId="5" r:id="R89fb77d077c2431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index Submissions" sheetId="6" r:id="R619889b9afa64214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18-Task Audit" sheetId="7" r:id="R625863f70a5f489e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="8" r:id="R05ff0594ac384509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider &amp; Address" sheetId="9" r:id="Rd7143bd93e254a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0785633b19df42c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Queries" sheetId="2" r:id="R7875c0bd7f624420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="3" r:id="R86db30b424824658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Countries" sheetId="4" r:id="Re9d7b3ccf92b4863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language Paths" sheetId="5" r:id="Ra657c7ba88cd4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index Submissions" sheetId="6" r:id="R352380f0db5d42d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18-Task Audit" sheetId="7" r:id="R55532faad3754363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="8" r:id="Rbd2506f6158245fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider &amp; Address" sheetId="9" r:id="R2003be1099cf4f8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17308,7 +17308,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b4d7d1535ad4c42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b90e118acf42c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17904,7 +17904,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d48c6bd6dc848b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc1c50a42424338"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19876,7 +19876,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e95f321e8404af1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0b4432d82b1486f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20261,13 +20261,13 @@
         <x:v>https://pelitparkhotel.com/ar/hotel-near-forum-trabzon/</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>Pending; inspected not indexed</x:v>
+        <x:v>Accepted 2026-09-11</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
         <x:v>In queue 2026-09-10 12:33</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>A retry did not show an acceptance confirmation; do not count as accepted.</x:v>
+        <x:v>Google inspection said not indexed before request; submission is not indexing.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -20290,7 +20290,7 @@
         <x:v>Processed/submitted does not prove indexing.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="14" t="str">
         <x:v>KTÜ Farabi</x:v>
       </x:c>
@@ -20301,16 +20301,16 @@
         <x:v>https://pelitparkhotel.com/farabi-hastanesi-yakin-otel/</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>Pending after Google quota</x:v>
+        <x:v>Accepted 2026-09-11</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
         <x:v>In queue 2026-09-10 12:33</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>Retry only after current status inspection and quota availability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+        <x:v>Google inspection said not indexed before request; submission is not indexing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="14" t="str">
         <x:v>KTÜ Farabi</x:v>
       </x:c>
@@ -20321,16 +20321,16 @@
         <x:v>https://pelitparkhotel.com/en/hotel-near-farabi-hospital/</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Pending after Google quota</x:v>
+        <x:v>Accepted 2026-09-11</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
         <x:v>In queue 2026-09-10 12:33</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>Retry only after current status inspection and quota availability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+        <x:v>Google inspection said not indexed before request; submission is not indexing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>KTÜ Farabi</x:v>
       </x:c>
@@ -20341,16 +20341,16 @@
         <x:v>https://pelitparkhotel.com/ar/hotel-near-farabi-hospital/</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Pending; not retried after quota</x:v>
+        <x:v>Accepted 2026-09-11</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
         <x:v>In queue 2026-09-10 12:33</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Retry only after current status inspection and quota availability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+        <x:v>Google inspection said not indexed before request; submission is not indexing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="14" t="str">
         <x:v>KTÜ Farabi</x:v>
       </x:c>
@@ -20361,13 +20361,13 @@
         <x:v>https://pelitparkhotel.com/ka/hotel-near-farabi-hospital/</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>Pending; not retried after quota</x:v>
+        <x:v>Indexed at inspection 2026-09-11; not resubmitted</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
         <x:v>Request processed 2026-09-09 12:49</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Retry only after current status inspection and quota availability.</x:v>
+        <x:v>Google showed the URL indexed with HTTPS and one valid breadcrumb item.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20376,7 +20376,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f05e1e52a9436e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re971056375f34059"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20720,10 +20720,10 @@
         <x:v>مكتمل جزئيًا</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>robots وsitemap وcanonical/hreflang محدثة؛ Yandex: 10 في الطابور و2 معالجة؛ Google: 7 طلبات مقبولة و5 معلقة.</x:v>
+        <x:v>robots وsitemap وcanonical/hreflang محدثة؛ Yandex: 10 في الطابور و2 معالجة؛ Google: 11 طلبًا مقبولًا، وصفحة فارابي الجورجية مفهرسة أصلًا ولم تُعد.</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>القبول/المعالجة لا يعني الفهرسة؛ راقب التغطية ولا تكرر الطلبات المقبولة.</x:v>
+        <x:v>القبول/المعالجة لا يعني الفهرسة؛ راقب التغطية ولا تكرر الطلبات المقبولة أو الصفحات المفهرسة.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" hidden="0" customHeight="1">
@@ -20792,7 +20792,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2635b0447764de8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e9239e6cfd14e38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21152,8 +21152,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82ad7d8aa59145d1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00157f3f6c994dfd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d6dd8b719384551"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R727cbf1d67da4922"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Document provider-managed hotel price connection
</commit_message>
<xml_diff>
--- a/outputs/seo-handover-2026-09-11/Pelit_Park_SEO_Baseline_and_Handover_2026-09-11.xlsx
+++ b/outputs/seo-handover-2026-09-11/Pelit_Park_SEO_Baseline_and_Handover_2026-09-11.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0785633b19df42c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Queries" sheetId="2" r:id="R7875c0bd7f624420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="3" r:id="R86db30b424824658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Countries" sheetId="4" r:id="Re9d7b3ccf92b4863"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language Paths" sheetId="5" r:id="Ra657c7ba88cd4168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index Submissions" sheetId="6" r:id="R352380f0db5d42d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18-Task Audit" sheetId="7" r:id="R55532faad3754363"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="8" r:id="Rbd2506f6158245fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider &amp; Address" sheetId="9" r:id="R2003be1099cf4f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3f62147e1d614819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Queries" sheetId="2" r:id="R1d6a9b06218d4513"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="3" r:id="R901c05a03d57465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Countries" sheetId="4" r:id="R3a039fc48bff453c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language Paths" sheetId="5" r:id="R9cf6b9f4beaf452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index Submissions" sheetId="6" r:id="Ra743a3463bae4769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18-Task Audit" sheetId="7" r:id="R8b55570aa6e04003"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="8" r:id="R490643644a514b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider &amp; Address" sheetId="9" r:id="R7ea6a8bf6bda4641"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17308,7 +17308,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b90e118acf42c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re74d96a70dc4452f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17904,7 +17904,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc1c50a42424338"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fdb573b570b4530"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19876,7 +19876,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0b4432d82b1486f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2da63d32f064cc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20376,7 +20376,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re971056375f34059"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re48c674b13094d58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20697,13 +20697,13 @@
         <x:v>Google Hotels</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>محجوب لدى المزود</x:v>
+        <x:v>مكتمل جزئيًا / يديره المزود</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>Google Hotels يعرض الفندق وأسعار بعض الشركاء، لكن ملكية اتصال Rezervasyonal/Hotel Center غير مثبتة من الحساب الحالي.</x:v>
+        <x:v>أكد مالك الفندق أن ElektraWeb/Rezervasyonal يرسل الأسعار إلى Google وأن موقع الفندق يحول الحجز إلى محرك المزود.</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>إرسال رسالة المزود وطلب Property ID وحالة feed وFree Booking Links والصلاحيات.</x:v>
+        <x:v>طلب حساب Hotel Center أو Property ID وحالة feed وFree Booking Links والصلاحيات، وربط حدث الحجز المكتمل.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
@@ -20792,7 +20792,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e9239e6cfd14e38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3e8c2d59f524050"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21152,8 +21152,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d6dd8b719384551"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R727cbf1d67da4922"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree3bf3b4ba764dbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98557677cecb465d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21196,12 +21196,12 @@
       <x:c r="E3" s="10"/>
       <x:c r="F3" s="10"/>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
+    <x:row r="4" ht="24" hidden="0" customHeight="1">
       <x:c r="A4" s="20" t="str">
-        <x:v>Website address</x:v>
+        <x:v>Booking provider</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>Üniversite Mh. Akif Saruhan Cd. No:77/1 Ortahisar / Trabzon</x:v>
+        <x:v>Owner-confirmed: ElektraWeb/Rezervasyonal supplies prices and availability to Google; pelitparkhotel.com sends booking users to https://pelit-park.rezervasyonal.com/.</x:v>
       </x:c>
       <x:c r="C4" s="14"/>
       <x:c r="D4" s="14"/>
@@ -21210,75 +21210,79 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>Google / Booking address</x:v>
+        <x:v>Website address</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Üniversite, Akif Saruhan Cd. No:77 (postal codes also differ across sources)</x:v>
+        <x:v>Üniversite Mh. Akif Saruhan Cd. No:77/1 Ortahisar / Trabzon</x:v>
       </x:c>
       <x:c r="C5" s="14"/>
       <x:c r="D5" s="14"/>
       <x:c r="E5" s="14"/>
       <x:c r="F5" s="14"/>
     </x:row>
-    <x:row r="6" ht="24" hidden="0" customHeight="1">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
-        <x:v>Authoritative source</x:v>
+        <x:v>Google / Booking address</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>Hotel operating licence, official municipal/UAVT address registration, or another current government-issued address record controlled by the hotel.</x:v>
+        <x:v>Üniversite, Akif Saruhan Cd. No:77 (postal codes also differ across sources)</x:v>
       </x:c>
       <x:c r="C6" s="14"/>
       <x:c r="D6" s="14"/>
       <x:c r="E6" s="14"/>
       <x:c r="F6" s="14"/>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
-        <x:v>Decision</x:v>
+        <x:v>Authoritative source</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>No correction proposed. Platform listings are secondary evidence and conflict; obtain the authoritative record first.</x:v>
+        <x:v>Hotel operating licence, official municipal/UAVT address registration, or another current government-issued address record controlled by the hotel.</x:v>
       </x:c>
       <x:c r="C7" s="14"/>
       <x:c r="D7" s="14"/>
       <x:c r="E7" s="14"/>
       <x:c r="F7" s="14"/>
     </x:row>
-    <x:row r="8" ht="24" hidden="0" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
-        <x:v>After confirmation</x:v>
+        <x:v>Decision</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>Update website structured data/footer, Google Business Profile, booking engine, Booking.com and other citations to the exact same NAP.</x:v>
+        <x:v>No correction proposed. Platform listings are secondary evidence and conflict; obtain the authoritative record first.</x:v>
       </x:c>
       <x:c r="C8" s="14"/>
       <x:c r="D8" s="14"/>
       <x:c r="E8" s="14"/>
       <x:c r="F8" s="14"/>
     </x:row>
-    <x:row r="9"/>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
+    <x:row r="9" ht="24" hidden="0" customHeight="1">
+      <x:c r="A9" s="20" t="str">
+        <x:v>After confirmation</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>Update website structured data/footer, Google Business Profile, booking engine, Booking.com and other citations to the exact same NAP.</x:v>
+      </x:c>
+      <x:c r="C9" s="14"/>
+      <x:c r="D9" s="14"/>
+      <x:c r="E9" s="14"/>
+      <x:c r="F9" s="14"/>
+    </x:row>
+    <x:row r="10"/>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="5" t="str">
         <x:v>Turkish message to ElektraWeb / Rezervasyonal</x:v>
       </x:c>
-      <x:c r="B10" s="5"/>
-      <x:c r="C10" s="5"/>
-      <x:c r="D10" s="5"/>
-      <x:c r="E10" s="5"/>
-      <x:c r="F10" s="5"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="14" t="str">
-        <x:v>Merhaba, Pelit Park Hotel (pelitparkhotel.com) için Rezervasyonal/ElektraWeb tarafında mevcut aktif bir Google Hotel Center bağlantısı ve Ücretsiz Rezervasyon Bağlantıları (Free Booking Links) entegrasyonu bulunuyor mu? Varsa bağlı Hotel Center hesabı veya Property ID’yi, fiyat/müsaitlik feed’inin son başarılı güncelleme durumunu ve erişim/yetki sürecini paylaşabilir misiniz? Bağlantı yoksa canlı fiyat ve müsaitliğin Google Hotels’e gönderilmesi için gerekli aktivasyon adımları, ücret/şartlar, teknik gereksinimler ve bizden istenen bilgiler nelerdir? Ayrıca doğrudan rezervasyon URL’sinin https://pelit-park.rezervasyonal.com/ olarak tanımlandığını teyit eder misiniz? Teşekkürler.</x:v>
-      </x:c>
-      <x:c r="B11" s="14"/>
-      <x:c r="C11" s="14"/>
-      <x:c r="D11" s="14"/>
-      <x:c r="E11" s="14"/>
-      <x:c r="F11" s="14"/>
+      <x:c r="B11" s="5"/>
+      <x:c r="C11" s="5"/>
+      <x:c r="D11" s="5"/>
+      <x:c r="E11" s="5"/>
+      <x:c r="F11" s="5"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="14"/>
+      <x:c r="A12" s="14" t="str">
+        <x:v>Merhaba, Pelit Park Hotel’in Rezervasyonal/ElektraWeb rezervasyon motorunun Google’a fiyat ve müsaitlik aktardığını ve pelitparkhotel.com üzerindeki rezervasyon bağlantılarının https://pelit-park.rezervasyonal.com/ adresine yönlendiğini teyit ediyoruz. Bağlı Google Hotel Center hesabını veya Property ID’yi, feed’in son başarılı güncelleme durumunu, Ücretsiz Rezervasyon Bağlantılarının (Free Booking Links) aktif olup olmadığını ve erişim/yetki sürecini paylaşabilir misiniz? Ayrıca tamamlanan rezervasyonları ölçmek için başarı sayfasında GTM/gtag olayı, postback/API veya başka bir dönüşüm entegrasyonu destekliyor musunuz? Varsa teknik dokümanı iletebilir misiniz? Teşekkürler.</x:v>
+      </x:c>
       <x:c r="B12" s="14"/>
       <x:c r="C12" s="14"/>
       <x:c r="D12" s="14"/>
@@ -21308,6 +21312,14 @@
       <x:c r="D15" s="14"/>
       <x:c r="E15" s="14"/>
       <x:c r="F15" s="14"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="14"/>
+      <x:c r="B16" s="14"/>
+      <x:c r="C16" s="14"/>
+      <x:c r="D16" s="14"/>
+      <x:c r="E16" s="14"/>
+      <x:c r="F16" s="14"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -21317,8 +21329,9 @@
     <x:mergeCell ref="B6:F6"/>
     <x:mergeCell ref="B7:F7"/>
     <x:mergeCell ref="B8:F8"/>
-    <x:mergeCell ref="A10:F10"/>
-    <x:mergeCell ref="A11:F15"/>
+    <x:mergeCell ref="B9:F9"/>
+    <x:mergeCell ref="A11:F11"/>
+    <x:mergeCell ref="A12:F16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>